<commit_message>
Add an optional "non-global files" field
Closes #166
</commit_message>
<xml_diff>
--- a/paired-tag/latest/paired-tag.xlsx
+++ b/paired-tag/latest/paired-tag.xlsx
@@ -119,6 +119,17 @@
     </comment>
     <comment ref="L1" authorId="1">
       <text>
+        <t>A semicolon separated list of non-shared files to be included in the dataset.
+The path assumes the files are located in the "TOP/non-global/" directory. For
+example, for the file is
+TOP/non-global/lab_processed/images/1-tissue-boundary.geojson the value of this
+field would be "./lab_processed/images/1-tissue-boundary.geojson". After ingest,
+these files will be copied to the appropriate locations within the respective
+dataset directory tree.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="1">
+      <text>
         <t>(Required) The unique string identifier for the metadata specification version,
 which is easily interpretable by computers for purposes of data validation and
 processing. Example: 22bc762a-5020-419d-b170-24253ed9e8d9</t>
@@ -129,7 +140,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="227">
   <si>
     <t>parent_sample_id</t>
   </si>
@@ -782,6 +793,9 @@
     <t>number_of_pre_amplification_pcr_cycles</t>
   </si>
   <si>
+    <t>non_global_files</t>
+  </si>
+  <si>
     <t>metadata_schema_id</t>
   </si>
   <si>
@@ -800,7 +814,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2026-06-29T15:40:39-07:00</t>
+    <t>2026-07-14T09:55:13-07:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -859,7 +873,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyAlignment="true" applyFill="true">
       <alignment horizontal="center"/>
@@ -876,6 +890,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -886,7 +901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" style="2" width="14.39453125" customWidth="true" bestFit="true"/>
@@ -900,7 +915,8 @@
     <col min="9" max="9" style="10" width="24.57421875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" style="11" width="21.765625" customWidth="true" bestFit="true"/>
     <col min="11" max="11" style="12" width="31.91796875" customWidth="true" bestFit="true"/>
-    <col min="12" max="12" style="13" width="16.91796875" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" style="13" width="13.33984375" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" style="14" width="16.91796875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -940,13 +956,16 @@
       <c r="L1" t="s" s="1">
         <v>217</v>
       </c>
+      <c r="M1" t="s" s="1">
+        <v>218</v>
+      </c>
     </row>
     <row r="2">
       <c r="D2" t="s" s="5">
         <v>112</v>
       </c>
-      <c r="L2" t="s" s="13">
-        <v>218</v>
+      <c r="M2" t="s" s="14">
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -1867,16 +1886,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2">
@@ -1884,13 +1903,13 @@
         <v>112</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new fields and value sets
Closes #169
Closes #170
Closes #171
Closes #172
</commit_message>
<xml_diff>
--- a/paired-tag/latest/paired-tag.xlsx
+++ b/paired-tag/latest/paired-tag.xlsx
@@ -8,10 +8,13 @@
   <sheets>
     <sheet name="Paired-Tag" r:id="rId3" sheetId="1"/>
     <sheet name="dataset_type" r:id="rId4" sheetId="2"/>
-    <sheet name="preparation_instrument_vendor" r:id="rId5" sheetId="3"/>
-    <sheet name="preparation_instrument_model" r:id="rId6" sheetId="4"/>
-    <sheet name="preparation_instrument_kit" r:id="rId7" sheetId="5"/>
-    <sheet name=".metadata" r:id="rId8" sheetId="6"/>
+    <sheet name="library_preparation_kit" r:id="rId5" sheetId="3"/>
+    <sheet name="preparation_instrument_vendor" r:id="rId6" sheetId="4"/>
+    <sheet name="preparation_instrument_model" r:id="rId7" sheetId="5"/>
+    <sheet name="preparation_instrument_kit" r:id="rId8" sheetId="6"/>
+    <sheet name="tag_enzyme_sequence" r:id="rId9" sheetId="7"/>
+    <sheet name="antibody_reagent_kit" r:id="rId10" sheetId="8"/>
+    <sheet name=".metadata" r:id="rId11" sheetId="9"/>
   </sheets>
 </workbook>
 </file>
@@ -76,6 +79,14 @@
     </comment>
     <comment ref="G1" authorId="1">
       <text>
+        <t>The reagent kit used to construct the sequencing library, including both the kit
+name and, if available, version and product number. If the library was prepared
+using a custom protocol, enter “Custom”. Example: 10X Genomics; Chromium Next
+GEM Single Cell 5' Kit v2, 16 rxns; PN 1000263</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="1">
+      <text>
         <t>(Required) A lab-assigned identifier used to indicate which cells or nuclei were
 captured together in the same run. For example, in a 10X Genomics Chromium
 Controller workflow, this could be the chip ID used to trace datasets derived
@@ -85,7 +96,7 @@
 Broad_Batch1234</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="1">
+    <comment ref="I1" authorId="1">
       <text>
         <t>(Required) The company that manufactures the instrument used to prepare the
 sample (e.g., for staining or other processing steps) prior to the assay. If the
@@ -93,7 +104,7 @@
 sample preparation occurred, enter "Not applicable". Example: 10X Genomics</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="1">
+    <comment ref="J1" authorId="1">
       <text>
         <t>(Required) The specific model of the instrument used for sample preparation,
 such as staining. Manufacturers may offer multiple models with varying features
@@ -102,7 +113,7 @@
 applicable". Example: Chromium X</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="1">
+    <comment ref="K1" authorId="1">
       <text>
         <t>(Required) The reagent kit used in conjunction with the preparation instrument
 for sample processing (e.g., staining or labeling). If the reagent kit was
@@ -110,14 +121,14 @@
 Chromium Next GEM Chip G Single Cell Kit, 48 rxns; PN 1000120</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="1">
+    <comment ref="L1" authorId="1">
       <text>
         <t>(Required) The number of PCR cycles performed following the Chromium Controller
 step and before the suspension is separated and library construction begins.
 Example: 7</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="1">
+    <comment ref="M1" authorId="1">
       <text>
         <t>A semicolon separated list of non-shared files to be included in the dataset.
 The path assumes the files are located in the "TOP/non-global/" directory. For
@@ -128,7 +139,26 @@
 dataset directory tree.</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="1">
+    <comment ref="N1" authorId="1">
+      <text>
+        <t>The unique two-nucleotide barcode sequence contained within the adapter
+introduced by the TAG Enzyme during tagmentation. In multiplexed Paired-Tag
+experiments, different tag enzyme sequences are assigned to different samples or
+assay conditions to distinguish them and are used to demultiplex the pooled
+sequencing data.</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="1">
+      <text>
+        <t>(Required) The antibody reagent used to recognize a specific protein target or
+histone modification during the Paired-Tag assay. These antibodies bind to their
+target epitopes and direct the tagmentation reaction to the corresponding
+chromatin regions, enabling profiling of chromatin features in individual cells.
+If a custom antibody reagent is used, then enter "Custom". Example: Abcam;
+Anti-Histone H3 (tri methyl K9) antibody [EPR16601] - ChIP Grade; PN: ab176916</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="1">
       <text>
         <t>(Required) The unique string identifier for the metadata specification version,
 which is easily interpretable by computers for purposes of data validation and
@@ -140,7 +170,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="324">
   <si>
     <t>parent_sample_id</t>
   </si>
@@ -508,6 +538,249 @@
     <t>data_path</t>
   </si>
   <si>
+    <t>library_preparation_kit</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' HT Kit v3.1, 8 rxns; PN 1000370</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000336</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Automated Single Cell 5' Kit v2, 4 rxns; PN 1000298</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000366</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell Fixed RNA Sample Preparation Kit, 16 rxns; PN 1000414</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000484</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium Spatial Gene Expression Slide and Reagent Kit, 4 slides, 16 reactions; PN 1000184</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000261</t>
+  </si>
+  <si>
+    <t>Parse Biosciences; Evercode WT v2 Kit, 48 rxns; PN ECW02030</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000341</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 5' Kit v2, 16 rxns; PN 1000263</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000339</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium Spatial for FFPE Gene Expression Kit, Human Transcriptome, 1 slides, 4 reactions; PN 1000338</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000320</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' Kit v3.1, 16 rxns; PN 1000268</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000337</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell ATAC Library &amp; Gel Bead Kit, 16 rxns; PN 1000175</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000471</t>
+  </si>
+  <si>
+    <t>10x Genomics; Library Construction Kit C, 16 rxns; PN 1000694</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000399</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Mouse Transcriptome, 6.5mm, 4 rxns; PN 1000521</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000432</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' HT Kit v3.1, 48 rxns; PN 1000348</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000335</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' GEM, Library &amp; Gel Bead Kit v3.1, 16 rxns; PN 1000121</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000334</t>
+  </si>
+  <si>
+    <t>10x Genomics; Library Construction Kit C, 4 rxns; PN 1000689</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000398</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Human Transcriptome, 11 mm, 2 reactions; PN 1000522</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000322</t>
+  </si>
+  <si>
+    <t>Illumina; TruSeq Stranded mRNA Library Prep (48 samples); PN 20020594</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000343</t>
+  </si>
+  <si>
+    <t>10X Genomics; Automated Library Construction Kit, 24 rxns; PN 1000428</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000374</t>
+  </si>
+  <si>
+    <t>New England BioLabs; NEBNext Ultra II RNA Library Prep Kit for Illumina; PN E7770</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000377</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Automated Single Cell 5' Kit v2, 24 rxns; PN 1000290</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000365</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium Spatial Gene Expression Slide and Reagent Kit, 1 slides, 4 reactions; PN 1000187</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000265</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium GEM-X Single Cell 5' Kit v3, 16 rxns; PN 1000699</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000394</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Single Cell ATAC Library &amp; Gel Bead Kit, 16 rxns; PN 1000110</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000469</t>
+  </si>
+  <si>
+    <t>10x Genomics; Library Construction Kit, 16 rxns; PN 1000190</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000439</t>
+  </si>
+  <si>
+    <t>Parse Biosciences; Evercode WT Mini v2 Kit, 12 rxns; PN ECW02010</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000342</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell 5' HT Kit v2, 48 rxns; PN 1000356</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000467</t>
+  </si>
+  <si>
+    <t>Illumina; TruSeq Stranded mRNA Library Prep (96 samples); PN 20020595</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000344</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 5' Kit v2, 4 rxns; PN 1000265</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000340</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 4 rxn; PN 1000285</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000251</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Hybridization &amp; Library Kit, 4 rxns; PN 1000415</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000375</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Single Cell 3' GEM, Library &amp; Gel Bead Kit v3, 4 rxns; PN 1000092</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000260</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Single Cell 3ʹ GEM, Library &amp; Gel Bead Kit v3, 16 rxns; PN 1000075</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000460</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Single Cell 3' Library &amp; Gel Bead Kit, 4 rxns; PN 120267</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000299</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium Spatial for FFPE Gene Expression Kit, Mouse Transcriptome, 4 rxns; PN 1000339</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000355</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 16 rxn; PN 1000283</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000250</t>
+  </si>
+  <si>
+    <t>Epigenome Technologies; Multiplex Droplet Paired-Tag 16 Reaction Kit; PN MDP16101</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000499</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' Kit v3.1, 4 rxns; PN 1000269</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000338</t>
+  </si>
+  <si>
+    <t>10x Genomics; GEM-X Flex GEM &amp; Library Kit, 4 rxns; PN 1000782</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000497</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell 5' HT Kit v2, 8 rxns; PN 1000374</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000466</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Human Transcriptome, 6.5mm, 4 reactions; PN 1000520</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000321</t>
+  </si>
+  <si>
     <t>capture_batch_id</t>
   </si>
   <si>
@@ -607,12 +880,6 @@
     <t>https://identifiers.org/RRID:SCR_019326</t>
   </si>
   <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
-  </si>
-  <si>
     <t>NanoZoomer S360</t>
   </si>
   <si>
@@ -706,12 +973,6 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000462</t>
   </si>
   <si>
-    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 4 rxn; PN 1000285</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000251</t>
-  </si>
-  <si>
     <t>10x Genomics; Visium HD, Mouse Transcriptome, 6.5 mm, 4 runs; PN 1000676</t>
   </si>
   <si>
@@ -754,12 +1015,6 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000379</t>
   </si>
   <si>
-    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 16 rxn; PN 1000283</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000250</t>
-  </si>
-  <si>
     <t>10x Genomics; Visium HD, Human Transcriptome, 11 mm, 4 runs; PN 1001037</t>
   </si>
   <si>
@@ -784,6 +1039,12 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000325</t>
   </si>
   <si>
+    <t>10x Genomics; GEM-X Flex Gene Expression Chip Kit, 4 chips; PN 1000791</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000498</t>
+  </si>
+  <si>
     <t>10x Genomics; Visium HD, Mouse Transcriptome, 11 mm, 4 runs; PN 1001038</t>
   </si>
   <si>
@@ -796,6 +1057,66 @@
     <t>non_global_files</t>
   </si>
   <si>
+    <t>tag_enzyme_sequence</t>
+  </si>
+  <si>
+    <t>GG</t>
+  </si>
+  <si>
+    <t>TT</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>antibody_reagent_kit</t>
+  </si>
+  <si>
+    <t>Standard BioTools; Maxpar Cytoplasmic/Secreted Antigen Staining Kit; PN 201602</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000410</t>
+  </si>
+  <si>
+    <t>Standard BioTools; Maxpar Cell Surface Staining Kit; PN 201601</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000411</t>
+  </si>
+  <si>
+    <t>Abcam; Anti-Histone H3 (tri methyl K9) antibody [EPR16601] - ChIP Grade; PN ab176916</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000502</t>
+  </si>
+  <si>
+    <t>Abcam; Anti-Histone H3 (acetyl K27) antibody [EP16602] - ChIP Grade; PN ab177178</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000501</t>
+  </si>
+  <si>
+    <t>Abcam; Anti-Histone H3 (tri methyl K27) antibody [mAbcam6002]- ChIP Grade; PN ab6002</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000500</t>
+  </si>
+  <si>
+    <t>Standard BioTools; Maxpar Nuclear Antigen Staining Kit; PN 201603</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000409</t>
+  </si>
+  <si>
+    <t>Standard BioTools; Maxpar Phosphoprotein Staining Kit; PN 201604</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000408</t>
+  </si>
+  <si>
     <t>metadata_schema_id</t>
   </si>
   <si>
@@ -814,7 +1135,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2026-07-14T09:55:13-07:00</t>
+    <t>2026-07-27T11:31:05-07:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -873,7 +1194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyAlignment="true" applyFill="true">
       <alignment horizontal="center"/>
@@ -888,7 +1209,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
@@ -901,7 +1225,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" style="2" width="14.39453125" customWidth="true" bestFit="true"/>
@@ -910,13 +1234,16 @@
     <col min="4" max="4" style="5" width="10.59765625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" style="6" width="14.5859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" style="7" width="8.46484375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" style="8" width="13.96484375" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" style="9" width="25.0859375" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" style="10" width="24.57421875" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" style="11" width="21.765625" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" style="12" width="31.91796875" customWidth="true" bestFit="true"/>
-    <col min="12" max="12" style="13" width="13.33984375" customWidth="true" bestFit="true"/>
-    <col min="13" max="13" style="14" width="16.91796875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" style="8" width="18.2734375" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" style="9" width="13.96484375" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" style="10" width="25.0859375" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" style="11" width="24.57421875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" style="12" width="21.765625" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" style="13" width="31.91796875" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" style="14" width="13.33984375" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" style="15" width="18.1015625" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" style="16" width="16.98828125" customWidth="true" bestFit="true"/>
+    <col min="16" max="16" style="17" width="16.91796875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -942,49 +1269,67 @@
         <v>122</v>
       </c>
       <c r="H1" t="s" s="1">
-        <v>123</v>
+        <v>203</v>
       </c>
       <c r="I1" t="s" s="1">
-        <v>146</v>
+        <v>204</v>
       </c>
       <c r="J1" t="s" s="1">
-        <v>183</v>
+        <v>227</v>
       </c>
       <c r="K1" t="s" s="1">
-        <v>216</v>
+        <v>262</v>
       </c>
       <c r="L1" t="s" s="1">
-        <v>217</v>
+        <v>293</v>
       </c>
       <c r="M1" t="s" s="1">
-        <v>218</v>
+        <v>294</v>
+      </c>
+      <c r="N1" t="s" s="1">
+        <v>295</v>
+      </c>
+      <c r="O1" t="s" s="1">
+        <v>300</v>
+      </c>
+      <c r="P1" t="s" s="1">
+        <v>315</v>
       </c>
     </row>
     <row r="2">
       <c r="D2" t="s" s="5">
         <v>112</v>
       </c>
-      <c r="M2" t="s" s="14">
-        <v>219</v>
+      <c r="P2" t="s" s="17">
+        <v>316</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="8">
     <dataValidation type="list" sqref="D2:D1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'dataset_type'!$A$1:$A$58</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="H2:H1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="G2:G1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'library_preparation_kit'!$A$1:$A$40</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'preparation_instrument_vendor'!$A$1:$A$11</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="J2:J1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'preparation_instrument_model'!$A$1:$A$19</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2:J1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'preparation_instrument_kit'!$A$1:$A$17</formula1>
+    <dataValidation type="list" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'preparation_instrument_kit'!$A$1:$A$18</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="between" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="whole" operator="between" sqref="L2:L1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="list" sqref="N2:N1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'tag_enzyme_sequence'!$A$1:$A$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="O2:O1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'antibody_reagent_kit'!$A$1:$A$8</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -1469,95 +1814,327 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="B1" t="s" s="0">
         <v>124</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>125</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s" s="0">
         <v>126</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>127</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="B3" t="s" s="0">
         <v>128</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>129</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="B4" t="s" s="0">
         <v>130</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>131</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="B5" t="s" s="0">
         <v>132</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>133</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="B6" t="s" s="0">
         <v>134</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>135</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>135</v>
+      </c>
+      <c r="B7" t="s" s="0">
         <v>136</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>137</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
+        <v>137</v>
+      </c>
+      <c r="B8" t="s" s="0">
         <v>138</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>139</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="B9" t="s" s="0">
         <v>140</v>
-      </c>
-      <c r="B9" t="s" s="0">
-        <v>141</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="B10" t="s" s="0">
         <v>142</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>143</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="B11" t="s" s="0">
         <v>144</v>
       </c>
-      <c r="B11" t="s" s="0">
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
         <v>145</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>149</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>151</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>153</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>155</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>163</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>165</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>169</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>171</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>181</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>183</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>185</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>187</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>193</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>195</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -1567,159 +2144,95 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>147</v>
+        <v>205</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>148</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>128</v>
+        <v>207</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>129</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>149</v>
+        <v>209</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>150</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>151</v>
+        <v>211</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>152</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>153</v>
+        <v>213</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>154</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>155</v>
+        <v>215</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>156</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>157</v>
+        <v>217</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>158</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>159</v>
+        <v>219</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>160</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>162</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>163</v>
+        <v>223</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>164</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>165</v>
+        <v>225</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>167</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>169</v>
-      </c>
-      <c r="B13" t="s" s="0">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="0">
-        <v>171</v>
-      </c>
-      <c r="B14" t="s" s="0">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="0">
-        <v>173</v>
-      </c>
-      <c r="B15" t="s" s="0">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>175</v>
-      </c>
-      <c r="B16" t="s" s="0">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="B17" t="s" s="0">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>179</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>181</v>
-      </c>
-      <c r="B19" t="s" s="0">
-        <v>182</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -1729,143 +2242,159 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>184</v>
+        <v>228</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>185</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>186</v>
+        <v>209</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>187</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>188</v>
+        <v>230</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>189</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>190</v>
+        <v>232</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>191</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>192</v>
+        <v>234</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>193</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>195</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>196</v>
+        <v>236</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>197</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>155</v>
+        <v>238</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>156</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>198</v>
+        <v>240</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>199</v>
+        <v>241</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>200</v>
+        <v>242</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>201</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>202</v>
+        <v>244</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>203</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>204</v>
+        <v>246</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>205</v>
+        <v>247</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>206</v>
+        <v>248</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>207</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>208</v>
+        <v>250</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>209</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>210</v>
+        <v>252</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>211</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>212</v>
+        <v>254</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>213</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>214</v>
+        <v>256</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>215</v>
+        <v>257</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -1874,6 +2403,264 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>265</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>269</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>271</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>273</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>181</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>275</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>281</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>285</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>287</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>289</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>291</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>292</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>299</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>305</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>309</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>181</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>314</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1886,16 +2673,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>220</v>
+        <v>317</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>221</v>
+        <v>318</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>223</v>
+        <v>320</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>225</v>
+        <v>322</v>
       </c>
     </row>
     <row r="2">
@@ -1903,13 +2690,13 @@
         <v>112</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>222</v>
+        <v>319</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>224</v>
+        <v>321</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>226</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>